<commit_message>
Complete IT sheet for MoFA Log - September 2026
Adds the Archive_2 emails and September WhatsApp items (IT now 24 rows).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TGjTRH6W5gZfxXYUTY19k1
</commit_message>
<xml_diff>
--- a/output/MoFA Log - September2026 Final.xlsx
+++ b/output/MoFA Log - September2026 Final.xlsx
@@ -21808,7 +21808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="5" min="1" max="1"/>
@@ -21909,24 +21909,727 @@
       </c>
       <c r="G3" s="7" t="n"/>
     </row>
-    <row r="4" ht="201" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="7" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="8" t="n">
+        <v>46271</v>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Request to Reposition and Reformat the Health Insurance Advisory Across UAE Traveller Pages</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+Following a previous request from the UAE Traveller team, the health insurance advisory below was added to the General Travel Guidelines section across all UAE Traveller destination pages.
+The sentence has already been added; however, it is currently displayed as the first item in the section. The UAE Traveller team has requested the following adjustments:
+- Move the sentence to the end of the General Travel Guidelines section.
+- Display it as a bullet point.
+- Ensure that its formatting and alignment are consistent with the other items in the section.
+- Apply the adjustment to both the Arabic and English versions across all destination pages.
+English text:
+It is advised to obtain valid international health insurance before traveling to cover any medical or healthcare needs that may arise during the trip.
+Arabic text:
+يُنصح بالحصول على تأمين صحي دولي ساري المفعول قبل السفر، لتغطية أي احتياجات صحية أو علاجية أثناء السفر.
+Example – UAE Traveller page for Brazil:
+https://www.mofa.gov.ae/en/travel-updates?code=BRA
+Please find the attached screenshot showing the sentence that requires repositioning and reformatting.
+We would appreciate your assistance in applying these changes across all relevant UAE Traveller destination pages and confirming once the update has been completed.
+Thank you once again for your continued support.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/en/travel-updates?code=BRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="306" customHeight="1">
+      <c r="A5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>46272</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update News Sections to the New Template – Islamabad and Accra Missions</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
+1. Islamabad Mission
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Islamabad/Media hub/News
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Islamabad/Media-hub/News
+2. Accra Mission
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Accra/Media hub/News
+News Section URL: https://www.mofa.gov.ae/Missions/_Inprogress/Accra/Media-hub/News
+We would appreciate your support in applying the new News section template to both missions while ensuring that all existing content, language versions, and related functionality are maintained correctly during the transition.
+Please let us know once the updates have been completed or if any additional information is required from our side.
+Thank you once again for your continued cooperation and support.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Islamabad/Media-hub/News</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="186" customHeight="1">
+      <c r="A6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>46272</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Request to Grant Viewer Access to Google Analytics (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srini
+We would like to kindly request your assistance, if possible, in adding the following email address to our Google Analytics account with Viewer access:
+ga4-83@sturdy-pivot-507908-t1.iam.gserviceaccount.com
+This access is needed to connect the Claude platform with Google Analytics, which will help enable faster reporting and more efficient data analysis.
+We would greatly appreciate it if you could grant this access at your earliest convenience. Please let me know if you need any further information from my side.
+Thank you very much for your time and support.
+(Srini's reply: please send to Kamal, he is the only one having the credentials.)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="231" customHeight="1">
+      <c r="A7" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update the News Section to the New Template – Zimbabwe Mission</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We kindly request your help in converting the News section of the UAE Mission website in Zimbabwe from the old template to the new approved News template.
+Please find the details below:
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Harare/Media hub/News
+Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Harare/Media-hub/News
+We would appreciate your support in applying the new template while ensuring that all existing news content and functionality are maintained correctly during the transition.
+Please let us know once the update has been completed or if any additional information is required from our side.
+Thank you once again for your continued support and cooperation.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Harare/Media-hub/News</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="246" customHeight="1">
+      <c r="A8" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Inquiry About Adding LinkedIn to the Social Media Section in the New Missions Template</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+Thank you very much for your continued support and assistance.
+Several missions, including Oslo and Helsinki, have requested the addition of their official LinkedIn account links to the Social Media section of their mission websites.
+Accordingly, we would appreciate your clarification on whether LinkedIn can be added as one of the supported social media platforms within the new missions template.
+If this option is currently supported, kindly advise us on the recommended method for adding and publishing the LinkedIn link through the CMS, including the relevant content path, field, or configuration that should be used.
+If LinkedIn is not currently available within the template, please let us know whether it can be enabled and whether any technical changes would be required from your side.
+Thank you in advance for your guidance and support.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="381" customHeight="1">
+      <c r="A9" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update News Sections to the New Template – Santiago and Podgorica Missions</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
+1. Santiago Mission – Republic of Chile
+Please apply the new News template to both the Arabic and English versions of the section.
+Arabic News Section URL: https://www.mofa.gov.ae/ar-ae/missions/_inprogress/santiago/media-hub/news
+English News Section URL: https://www.mofa.gov.ae/en/missions/_inprogress/santiago/media-hub/news
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Santiago/Media hub/News
+2. Podgorica Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Podgorica
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Podgorica/Media hub/News
+We would appreciate your support in applying the new approved template to the News sections of both missions, while ensuring that all existing news content, language versions, links, and functionality are retained correctly during the transition.
+Please let us know once the updates have been completed or if any additional information is required from our side.
+Thank you once again for your continued support and cooperation.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/missions/_inprogress/santiago/media-hub/news</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/en/missions/_inprogress/santiago/media-hub/news</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="321" customHeight="1">
+      <c r="A10" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update the Hebrew Title of the Ambassador Page – Tel Aviv Mission</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We kindly request your assistance in updating the Hebrew title of the Ambassador page on the UAE Mission website in Tel Aviv.
+Please replace the current title:
+הקונסול הכללי
+with the following title:
+השגריר
+We attempted to update the title through the relevant dictionary entry in the CMS; however, the change was not reflected on the website.
+Dictionary Path:
+/sitecore/content/LDSC/Global/Dictionary/Missions Website/About Embassy/The Ambassador
+Affected Page URL:
+https://www.mofa.gov.ae/he-il/Missions/_Inprogress/Tel-Aviv/The-Embassy/About-the-Consul
+Please find the attached screenshot showing the location of the title that needs to be updated.
+We would appreciate your support in reviewing the issue and applying the requested title change to the Hebrew version of the page.
+Thank you very much for your continued support and assistance.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/he-il/Missions/_Inprogress/Tel-Aviv/The-Embassy/About-the-Consul</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="246" customHeight="1">
+      <c r="A11" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update Hebrew Text Direction to Right-to-Left – Tel Aviv Mission Website</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+Based on the instructions received from the UAE Mission in Tel Aviv, we kindly request your assistance in updating the text direction of the Hebrew-language content across the mission website.
+The Hebrew text is currently displayed from left to right (LTR). As Hebrew is a right-to-left language, please update the website configuration so that all Hebrew text, content components, and page elements are displayed from right to left (RTL), consistent with the Arabic version.
+Mission Website:
+https://www.mofa.gov.ae/he-il/Missions/_Inprogress/Tel-Aviv
+We would appreciate your support in reviewing the entire Hebrew version to ensure that the text direction, alignment, menus, and related interface elements are displayed correctly across both desktop and mobile devices.
+Please confirm once the requested update has been completed.
+Thank you very much for your continued support and assistance.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/he-il/Missions/_Inprogress/Tel-Aviv</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="409" customHeight="1">
+      <c r="A12" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update News Sections to the New Template – Multiple Missions</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
+1. Rome Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/rome
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Rome/Media hub/News
+2. Prague Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Prague
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Prague/Media hub/News
+3. Lisbon Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/lisbon
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Lisbon/Media hub/Embassy News
+4. Conakry Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Conakry/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Conakry/Media hub/News
+5. Colombo Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/missions/_inprogress/colombo/media-hub/news
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Colombo/Media hub/News
+We would appreciate your support in applying the new approved News template to all the above mission websites, while ensuring that the existing news content, links, and related functionality are maintained correctly during the transition.
+Please let us know once the updates have been completed or if any additional information or action is required from our side.
+Thank you once again for your continued support and cooperation.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/rome</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="409" customHeight="1">
+      <c r="A13" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Request to Centralize Contact Information Across Mission Website Pages</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan
+We would appreciate your support in reviewing a recurring issue we have noticed in the CMS, where certain contact details need to be entered separately in more than one location across the mission website.
+The duplicated information includes:
+- Phone number
+- Email address
+- Emergency number
+- Address
+Please find attached two screenshots for clarification. The screenshots are taken from the Jakarta Mission website.
+About the Embassy Page:
+https://www.mofa.gov.ae/Missions/Jakarta/The-Embassy/About-the-Consul
+The embassy information is displayed on the mission homepage as well as on the relevant embassy/ambassador page.
+Contact List Page:
+https://www.mofa.gov.ae/Missions/Jakarta/Contact-Form
+To improve consistency and reduce the risk of data mismatches, we would like to ask whether it is possible to configure these contact details so that they are entered only once in the CMS and automatically reflected across the other relevant pages.
+This would help simplify the publishing process, avoid duplicate data entry, and ensure that any future updates are applied consistently across the website.
+We would appreciate your advice on whether this can be implemented and, if so, the recommended approach.
+Thank you very much for your continued support and assistance.
+Regards,
+(Attachments: a.png, b.png)</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/Missions/Jakarta/The-Embassy/About-the-Consul</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="409" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Request to Remove Two Statements from the Digital Attestation Page Across All Mission Websites</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+Based on a request from Carla from the Government Communication Department, we kindly ask for your support in removing two statements from the Digital Attestation page across all mission websites, in both the Arabic and English versions.
+Please find below the statements that need to be removed:
+Arabic:
+- إجراءات رقمية شاملة: تقديم واستلام وثيقة التصديق إلكترونيًا.
+- خدمة سريعة: تتم عملية التصديق في غضون 2-3 أيام عمل.
+English:
+- Fully Digital Workflow: Submit and receive attested documents entirely online.
+- Faster Processing: Most requests are completed within 2–3 business days.
+Please also find attached two screenshots highlighting the exact statements to be removed in both languages.
+For reference, below are example links from the Muscat Mission website:
+Arabic: https://www.mofa.gov.ae/ar-ae/Missions/Muscat/Services/Services-for-Individuals/Attestation-Information
+English: https://www.mofa.gov.ae/en/Missions/Muscat/Services/Services-for-Individuals/Attestation-Information
+We would appreciate your support in applying this update consistently across all mission websites where the Digital Attestation page is available.
+Please let us know once the update has been completed or if any further information is required from our side.
+Thank you very much for your continued support and assistance.
+Regards,
+(Attachments: en[23].png, ar[89].png)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/Muscat/Services/Services-for-Individuals/Attestation-Information</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/en/Missions/Muscat/Services/Services-for-Individuals/Attestation-Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="409" customHeight="1">
+      <c r="A15" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update News Sections to the New Template – Multiple Missions</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+Thank you very much for your continued support and assistance.
+We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
+1. Ngerulmud Mission – Palau
+News Section URL: https://www.mofa.gov.ae/en/Missions/_Inprogress/Ngerulmud/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Ngerulmud/Media hub/News
+Important Note:
+For clarification, we have also noticed that when a new news item is created for any mission, it is currently generated automatically using the old News template, rather than the new approved template.
+We would appreciate your support in reviewing this behavior as well, so that newly created news items use the new template by default.
+2. Stockholm Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Stockholm/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Stockholm/Media hub/News
+3. Dublin Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Dublin/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Dublin/Media hub/News
+4. Kabul Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Kabul
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Kabul/Media hub/News
+5. Los Angeles Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Los-Angeles/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Los Angeles/Media hub/News
+We would appreciate your support in applying the new approved News template to all the above mission websites, while ensuring that the existing news content and functionality remain intact during the transition.
+In addition, kindly review the default behavior for creating new news items across mission websites, so that all future news items are created using the new template automatically.
+Please let us know once the updates have been completed or if any additional information is required from our side.
+Thank you once again for your continued support and cooperation.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Stockholm/Media-hub/News</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/en/Missions/_Inprogress/Ngerulmud/Media-hub/News</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="409" customHeight="1">
+      <c r="A16" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Request to Migrate News Sections to the New Approved Template – Multiple Missions</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We kindly request your help in migrating the News sections from the old template to the new approved News template for the following mission websites:
+1. Houston Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Houston/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Houston/Media hub/News
+2. Damascus Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/missions/_inprogress/damascus/media-hub/news
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Damascus/Media hub/News
+3. Geneva Consulate
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Geneva-Consulate/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Geneva-Consulate/Media hub/News
+4. Nairobi Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Nairobi
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Nairobi/Media hub/News
+5. Nouakchott Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Nouakchott
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Nouakchott/Media hub/News
+6. Kuala Lumpur Mission
+Mission Website URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Kuala-Lumpur
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Kuala Lumpur/Media hub/News
+We would appreciate your support in applying the new approved News template to the above mission websites while ensuring that all existing content, links, language versions, media assets, and related functionality are preserved correctly during the transition.
+Please let us know once the updates have been completed or if any additional information or action is required from our side.
+Thank you once again for your continued support and cooperation.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Houston/Media-hub/News</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="n"/>
+    </row>
+    <row r="17" ht="366" customHeight="1">
+      <c r="A17" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Homepage Display Issue – Banner Images and Welcome Message</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+While implementing some recent updates, we noticed a display issue affecting the homepage layout, specifically the main banner and the Welcome Message section.
+The issues observed are as follows:
+- The banner image does not fully cover the entire banner area.
+- When more than one banner image is configured, all images appear at the same time instead of displaying correctly as separate slides.
+- The Welcome Message appears larger than expected, causing parts of the text to be cut off or hidden.
+Please find below two examples where the issue can currently be observed:
+Victoria Mission: https://www.mofa.gov.ae/en/Missions/victoria
+Ankara Mission: https://www.mofa.gov.ae/en/Missions/Ankara
+A screenshot from the Victoria Mission website is also attached for reference.
+We would appreciate your support in reviewing the homepage component and resolving these display issues, while ensuring that:
+- banner images properly fit and cover the designated area,
+- multiple banner images rotate/display correctly,
+- and the Welcome Message is displayed at the appropriate size without any content being truncated.
+Thank you very much for your continued support and assistance.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/en/Missions/victoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="201" customHeight="1">
+      <c r="A18" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Re: Homepage Display Issue – Banner Images and Welcome Message</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+Thank you again for your continued support.
+I wanted to kindly follow up on the request below, as we have noticed that the same issue is now appearing across several mission websites, particularly in relation to the homepage banner and Welcome Message display.
+We have also started receiving emails from the missions regarding this issue, so we would appreciate it if you could advise whether there is an estimated timeline for resolving it.
+Having an expected timeframe would help us respond to the missions accordingly and manage their expectations until the issue is resolved.
+Thank you very much for your support and assistance.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="171" customHeight="1">
+      <c r="A19" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Re: Homepage Display Issue – Banner Images and Welcome Message</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We have now applied the recommended action and cleared the cache. As shown in the attached screenshot, the banner images are now displaying correctly.
+However, the issue with the Welcome Message title and text has reappeared. The font size has returned to the larger size, causing part of the Welcome Message to be cut off and preventing the full content from being displayed.
+Based on this behavior, we believe there may still be an underlying technical issue affecting the Welcome Message component.
+Could you please review this further and advise on the permanent solution?
+Thank you very much for your continued support and assistance.
+Regards,</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="156" customHeight="1">
+      <c r="A20" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Urgent: Ministry Website and CMS Completely Down (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Sorry for the inconvenience, Srini, but this is an urgent and critical matter.
+The Ministry's website &amp; CMS also is currently down and appears to be completely offline. None of the pages are accessible, and the entire website is not functioning.
+Could you please look into this issue and resolve it as soon as possible? The website is currently completely unavailable.
+Thank you for your urgent support.
+(Screenshots attached)
+Update (1:27 AM): Working now.</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="201" customHeight="1">
+      <c r="A21" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="8" t="n">
         <v>46292</v>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Request to Add Amharic Language to the CMS – Addis Ababa Mission</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Based on a request from the UAE Mission in Addis Ababa, and following approval from Nasra from the Government Communication Department, we kindly request your support in adding Amharic as an available language within the CMS for the Addis Ababa Mission website.
@@ -21936,27 +22639,80 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="336" customHeight="1">
-      <c r="A5" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="8" t="n">
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="409" customHeight="1">
+      <c r="A22" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>46292</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Request to Update News Sections to the New Template – Multiple Mission Websites</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Hi Srinivasan,
+We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
+1. Tashkent Mission
+Mission Website: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Tashkent
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Tashkent/Media hub/News
+2. Warsaw Mission
+Mission Website: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Warsaw
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Warsaw/Media hub/News
+3. Bucharest Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Bucharest/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Bucharest/Media hub/News
+4. Zanzibar Mission
+Mission Website: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Zanzibar
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Zanzibar/Media hub/News
+5. Dhaka Mission
+Mission Website: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Dhaka
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Dhaka/Media hub/News
+6. Geneva Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Geneva/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Geneva/Media hub/News
+7. Boston Mission
+News Section URL: https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Boston/Media-hub/News
+Sitecore Path: /sitecore/content/LDSC/Home/Missions/_Inprogress/Boston/Media hub/News
+8. Astana Mission
+(The rest of the email is not visible in the screenshot.)</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Tashkent</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="336" customHeight="1">
+      <c r="A23" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="8" t="n">
         <v>46293</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Request to Fix Navigation Menu Hover Behavior on Mission Websites</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We would like to bring to your attention an issue affecting the navigation menu on the mission websites.
@@ -21972,31 +22728,31 @@
 (Attachment: WhatsApp Video – 2.6 MB)</t>
         </is>
       </c>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/missions/Sao-Paulo</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="409" customHeight="1">
-      <c r="A6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="8" t="n">
+    <row r="24" ht="409" customHeight="1">
+      <c r="A24" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="8" t="n">
         <v>46294</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Request to Update News Sections to the New Template – Multiple Mission Websites</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 We kindly request your help in converting the News sections from the old template to the new approved News template for the following mission websites:
@@ -22021,35 +22777,35 @@
 Regards,</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/ar-ae/Missions/_Inprogress/Kampala</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>https://www.mofa.gov.ae/en/Missions/_Inprogress/Addis-Ababa</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="111" customHeight="1">
-      <c r="A7" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="8" t="n">
+    <row r="25" ht="111" customHeight="1">
+      <c r="A25" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="8" t="n">
         <v>46294</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Country name issue</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>(Received from Srinivasan K – MoFA IT)
 Hi Team - Please update the Arabic name for this country, as the country name is currently displayed in English on the Arabic Attestation Service.
@@ -22058,27 +22814,27 @@
 Srini</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="336" customHeight="1">
-      <c r="A8" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="8" t="n">
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="336" customHeight="1">
+      <c r="A26" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="8" t="n">
         <v>46295</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Re: Country name issue</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Hi Srinivasan,
 Regarding the country name displayed on the UAE Traveller website, we have noticed that "French Guiana" currently appears in English on both the English and Arabic versions of the website. This indicates that no Arabic name has been configured for the country in the system.
@@ -22093,27 +22849,9 @@
 (Attachment: 18-11-2025.png)</t>
         </is>
       </c>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-    </row>
-    <row r="9" ht="156" customHeight="1"/>
-    <row r="10" ht="306" customHeight="1"/>
-    <row r="11" ht="216" customHeight="1"/>
-    <row r="12" ht="396" customHeight="1"/>
-    <row r="13" ht="171" customHeight="1"/>
-    <row r="14" ht="351" customHeight="1"/>
-    <row r="15" ht="336" customHeight="1"/>
-    <row r="16" ht="171" customHeight="1"/>
-    <row r="17" ht="321" customHeight="1"/>
-    <row r="18" ht="186" customHeight="1"/>
-    <row r="19" ht="201" customHeight="1"/>
-    <row r="20" ht="201" customHeight="1"/>
-    <row r="21" ht="306" customHeight="1"/>
-    <row r="22" ht="201" customHeight="1"/>
-    <row r="23" ht="201" customHeight="1"/>
-    <row r="24" ht="231" customHeight="1"/>
-    <row r="25" ht="126" customHeight="1"/>
-    <row r="26" ht="216" customHeight="1"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+    </row>
     <row r="27" ht="171" customHeight="1"/>
     <row r="28" ht="231" customHeight="1"/>
     <row r="29" ht="409" customHeight="1"/>
@@ -22158,9 +22896,25 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>